<commit_message>
fix: close phase 1 compatibility gaps
</commit_message>
<xml_diff>
--- a/dist/xlsx/cities-filtered.xlsx
+++ b/dist/xlsx/cities-filtered.xlsx
@@ -15781,33 +15781,33 @@
     </row>
     <row r="770">
       <c r="A770">
-        <v>10300010002401</v>
+        <v>10300010002144</v>
       </c>
       <c r="B770" t="str">
-        <v>آقکند</v>
+        <v>ترکمانچای</v>
       </c>
       <c r="C770" t="str">
-        <v>آقکند</v>
+        <v>ترکمانچای</v>
       </c>
       <c r="D770">
         <v>103</v>
       </c>
       <c r="E770">
-        <v>10300010</v>
+        <v>10300029</v>
       </c>
       <c r="F770">
-        <v>10300010002</v>
+        <v>10300029001</v>
       </c>
     </row>
     <row r="771">
       <c r="A771">
-        <v>10300010002402</v>
+        <v>10300010002401</v>
       </c>
       <c r="B771" t="str">
-        <v>ترک</v>
+        <v>آقکند</v>
       </c>
       <c r="C771" t="str">
-        <v>ترک</v>
+        <v>آقکند</v>
       </c>
       <c r="D771">
         <v>103</v>
@@ -15816,18 +15816,18 @@
         <v>10300010</v>
       </c>
       <c r="F771">
-        <v>10300010003</v>
+        <v>10300010002</v>
       </c>
     </row>
     <row r="772">
       <c r="A772">
-        <v>10300010002842</v>
+        <v>10300010002402</v>
       </c>
       <c r="B772" t="str">
-        <v>اچاچی</v>
+        <v>ترک</v>
       </c>
       <c r="C772" t="str">
-        <v>اچاچی</v>
+        <v>ترک</v>
       </c>
       <c r="D772">
         <v>103</v>
@@ -15836,38 +15836,38 @@
         <v>10300010</v>
       </c>
       <c r="F772">
-        <v>10300010004</v>
+        <v>10300010003</v>
       </c>
     </row>
     <row r="773">
       <c r="A773">
-        <v>10300011001234</v>
+        <v>10300010002842</v>
       </c>
       <c r="B773" t="str">
-        <v>هشترود</v>
+        <v>اچاچی</v>
       </c>
       <c r="C773" t="str">
-        <v>هشترود</v>
+        <v>اچاچی</v>
       </c>
       <c r="D773">
         <v>103</v>
       </c>
       <c r="E773">
-        <v>10300011</v>
+        <v>10300010</v>
       </c>
       <c r="F773">
-        <v>10300011002</v>
+        <v>10300010004</v>
       </c>
     </row>
     <row r="774">
       <c r="A774">
-        <v>10300011002590</v>
+        <v>10300011001234</v>
       </c>
       <c r="B774" t="str">
-        <v>نظرکهریزی</v>
+        <v>هشترود</v>
       </c>
       <c r="C774" t="str">
-        <v>نظرکهریزی</v>
+        <v>هشترود</v>
       </c>
       <c r="D774">
         <v>103</v>
@@ -15876,78 +15876,78 @@
         <v>10300011</v>
       </c>
       <c r="F774">
-        <v>10300011003</v>
+        <v>10300011002</v>
       </c>
     </row>
     <row r="775">
       <c r="A775">
-        <v>10300012001221</v>
+        <v>10300011002590</v>
       </c>
       <c r="B775" t="str">
-        <v>بناب</v>
+        <v>نظرکهریزی</v>
       </c>
       <c r="C775" t="str">
-        <v>بناب</v>
+        <v>نظرکهریزی</v>
       </c>
       <c r="D775">
         <v>103</v>
       </c>
       <c r="E775">
-        <v>10300012</v>
+        <v>10300011</v>
       </c>
       <c r="F775">
-        <v>10300012001</v>
+        <v>10300011003</v>
       </c>
     </row>
     <row r="776">
       <c r="A776">
-        <v>10300013001025</v>
+        <v>10300012001221</v>
       </c>
       <c r="B776" t="str">
-        <v>کردکندی</v>
+        <v>بناب</v>
       </c>
       <c r="C776" t="str">
-        <v>کردکندی</v>
+        <v>بناب</v>
       </c>
       <c r="D776">
         <v>103</v>
       </c>
       <c r="E776">
-        <v>10300013</v>
+        <v>10300012</v>
       </c>
       <c r="F776">
-        <v>10300013002</v>
+        <v>10300012001</v>
       </c>
     </row>
     <row r="777">
       <c r="A777">
-        <v>10300014001083</v>
+        <v>10300013001025</v>
       </c>
       <c r="B777" t="str">
-        <v>نظرلو</v>
+        <v>کردکندی</v>
       </c>
       <c r="C777" t="str">
-        <v>نظرلو</v>
+        <v>کردکندی</v>
       </c>
       <c r="D777">
         <v>103</v>
       </c>
       <c r="E777">
-        <v>10300014</v>
+        <v>10300013</v>
       </c>
       <c r="F777">
-        <v>10300014001</v>
+        <v>10300013002</v>
       </c>
     </row>
     <row r="778">
       <c r="A778">
-        <v>10300014001208</v>
+        <v>10300014001083</v>
       </c>
       <c r="B778" t="str">
-        <v>تسوج</v>
+        <v>نظرلو</v>
       </c>
       <c r="C778" t="str">
-        <v>تسوج</v>
+        <v>نظرلو</v>
       </c>
       <c r="D778">
         <v>103</v>
@@ -15956,18 +15956,18 @@
         <v>10300014</v>
       </c>
       <c r="F778">
-        <v>10300014003</v>
+        <v>10300014001</v>
       </c>
     </row>
     <row r="779">
       <c r="A779">
-        <v>10300014001209</v>
+        <v>10300014001208</v>
       </c>
       <c r="B779" t="str">
-        <v>خامنه</v>
+        <v>تسوج</v>
       </c>
       <c r="C779" t="str">
-        <v>خامنه</v>
+        <v>تسوج</v>
       </c>
       <c r="D779">
         <v>103</v>
@@ -15976,18 +15976,18 @@
         <v>10300014</v>
       </c>
       <c r="F779">
-        <v>10300014002</v>
+        <v>10300014003</v>
       </c>
     </row>
     <row r="780">
       <c r="A780">
-        <v>10300014001210</v>
+        <v>10300014001209</v>
       </c>
       <c r="B780" t="str">
-        <v>شبستر</v>
+        <v>خامنه</v>
       </c>
       <c r="C780" t="str">
-        <v>شبستر</v>
+        <v>خامنه</v>
       </c>
       <c r="D780">
         <v>103</v>
@@ -16001,13 +16001,13 @@
     </row>
     <row r="781">
       <c r="A781">
-        <v>10300014001211</v>
+        <v>10300014001210</v>
       </c>
       <c r="B781" t="str">
-        <v>شرفخانه</v>
+        <v>شبستر</v>
       </c>
       <c r="C781" t="str">
-        <v>شرفخانه</v>
+        <v>شبستر</v>
       </c>
       <c r="D781">
         <v>103</v>
@@ -16021,13 +16021,13 @@
     </row>
     <row r="782">
       <c r="A782">
-        <v>10300014001212</v>
+        <v>10300014001211</v>
       </c>
       <c r="B782" t="str">
-        <v>صوفیان</v>
+        <v>شرفخانه</v>
       </c>
       <c r="C782" t="str">
-        <v>صوفیان</v>
+        <v>شرفخانه</v>
       </c>
       <c r="D782">
         <v>103</v>
@@ -16036,18 +16036,18 @@
         <v>10300014</v>
       </c>
       <c r="F782">
-        <v>10300014001</v>
+        <v>10300014002</v>
       </c>
     </row>
     <row r="783">
       <c r="A783">
-        <v>10300014002101</v>
+        <v>10300014001212</v>
       </c>
       <c r="B783" t="str">
-        <v>شندآباد</v>
+        <v>صوفیان</v>
       </c>
       <c r="C783" t="str">
-        <v>شندآباد</v>
+        <v>صوفیان</v>
       </c>
       <c r="D783">
         <v>103</v>
@@ -16056,18 +16056,18 @@
         <v>10300014</v>
       </c>
       <c r="F783">
-        <v>10300014002</v>
+        <v>10300014001</v>
       </c>
     </row>
     <row r="784">
       <c r="A784">
-        <v>10300014002148</v>
+        <v>10300014002101</v>
       </c>
       <c r="B784" t="str">
-        <v>سیس</v>
+        <v>شندآباد</v>
       </c>
       <c r="C784" t="str">
-        <v>سیس</v>
+        <v>شندآباد</v>
       </c>
       <c r="D784">
         <v>103</v>
@@ -16081,13 +16081,13 @@
     </row>
     <row r="785">
       <c r="A785">
-        <v>10300014002149</v>
+        <v>10300014002148</v>
       </c>
       <c r="B785" t="str">
-        <v>وایقان</v>
+        <v>سیس</v>
       </c>
       <c r="C785" t="str">
-        <v>وایقان</v>
+        <v>سیس</v>
       </c>
       <c r="D785">
         <v>103</v>
@@ -16101,13 +16101,13 @@
     </row>
     <row r="786">
       <c r="A786">
-        <v>10300014002946</v>
+        <v>10300014002149</v>
       </c>
       <c r="B786" t="str">
-        <v>داریان</v>
+        <v>وایقان</v>
       </c>
       <c r="C786" t="str">
-        <v>داریان</v>
+        <v>وایقان</v>
       </c>
       <c r="D786">
         <v>103</v>
@@ -16121,13 +16121,13 @@
     </row>
     <row r="787">
       <c r="A787">
-        <v>10300014002947</v>
+        <v>10300014002946</v>
       </c>
       <c r="B787" t="str">
-        <v>علیشاه</v>
+        <v>داریان</v>
       </c>
       <c r="C787" t="str">
-        <v>علیشاه</v>
+        <v>داریان</v>
       </c>
       <c r="D787">
         <v>103</v>
@@ -16141,53 +16141,53 @@
     </row>
     <row r="788">
       <c r="A788">
-        <v>10300015001199</v>
+        <v>10300014002947</v>
       </c>
       <c r="B788" t="str">
-        <v>کلیبر</v>
+        <v>علیشاه</v>
       </c>
       <c r="C788" t="str">
-        <v>کلیبر</v>
+        <v>علیشاه</v>
       </c>
       <c r="D788">
         <v>103</v>
       </c>
       <c r="E788">
-        <v>10300015</v>
+        <v>10300014</v>
       </c>
       <c r="F788">
-        <v>10300015002</v>
+        <v>10300014002</v>
       </c>
     </row>
     <row r="789">
       <c r="A789">
-        <v>10300016001217</v>
+        <v>10300015001199</v>
       </c>
       <c r="B789" t="str">
-        <v>هریس</v>
+        <v>کلیبر</v>
       </c>
       <c r="C789" t="str">
-        <v>هریس</v>
+        <v>کلیبر</v>
       </c>
       <c r="D789">
         <v>103</v>
       </c>
       <c r="E789">
-        <v>10300016</v>
+        <v>10300015</v>
       </c>
       <c r="F789">
-        <v>10300016002</v>
+        <v>10300015002</v>
       </c>
     </row>
     <row r="790">
       <c r="A790">
-        <v>10300016002146</v>
+        <v>10300016001217</v>
       </c>
       <c r="B790" t="str">
-        <v>خواجه</v>
+        <v>هریس</v>
       </c>
       <c r="C790" t="str">
-        <v>خواجه</v>
+        <v>هریس</v>
       </c>
       <c r="D790">
         <v>103</v>
@@ -16196,18 +16196,18 @@
         <v>10300016</v>
       </c>
       <c r="F790">
-        <v>10300016001</v>
+        <v>10300016002</v>
       </c>
     </row>
     <row r="791">
       <c r="A791">
-        <v>10300016002147</v>
+        <v>10300016002146</v>
       </c>
       <c r="B791" t="str">
-        <v>زرنق</v>
+        <v>خواجه</v>
       </c>
       <c r="C791" t="str">
-        <v>زرنق</v>
+        <v>خواجه</v>
       </c>
       <c r="D791">
         <v>103</v>
@@ -16216,18 +16216,18 @@
         <v>10300016</v>
       </c>
       <c r="F791">
-        <v>10300016002</v>
+        <v>10300016001</v>
       </c>
     </row>
     <row r="792">
       <c r="A792">
-        <v>10300016002230</v>
+        <v>10300016002147</v>
       </c>
       <c r="B792" t="str">
-        <v>بخشایش</v>
+        <v>زرنق</v>
       </c>
       <c r="C792" t="str">
-        <v>بخشایش</v>
+        <v>زرنق</v>
       </c>
       <c r="D792">
         <v>103</v>
@@ -16241,13 +16241,13 @@
     </row>
     <row r="793">
       <c r="A793">
-        <v>10300016002333</v>
+        <v>10300016002230</v>
       </c>
       <c r="B793" t="str">
-        <v>کلوانق</v>
+        <v>بخشایش</v>
       </c>
       <c r="C793" t="str">
-        <v>کلوانق</v>
+        <v>بخشایش</v>
       </c>
       <c r="D793">
         <v>103</v>
@@ -16261,13 +16261,13 @@
     </row>
     <row r="794">
       <c r="A794">
-        <v>10300016002935</v>
+        <v>10300016002333</v>
       </c>
       <c r="B794" t="str">
-        <v>اربطان</v>
+        <v>کلوانق</v>
       </c>
       <c r="C794" t="str">
-        <v>اربطان</v>
+        <v>کلوانق</v>
       </c>
       <c r="D794">
         <v>103</v>
@@ -16276,38 +16276,38 @@
         <v>10300016</v>
       </c>
       <c r="F794">
-        <v>10300016001</v>
+        <v>10300016002</v>
       </c>
     </row>
     <row r="795">
       <c r="A795">
-        <v>10300019001225</v>
+        <v>10300016002935</v>
       </c>
       <c r="B795" t="str">
-        <v>جلفا</v>
+        <v>اربطان</v>
       </c>
       <c r="C795" t="str">
-        <v>جلفا</v>
+        <v>اربطان</v>
       </c>
       <c r="D795">
         <v>103</v>
       </c>
       <c r="E795">
-        <v>10300019</v>
+        <v>10300016</v>
       </c>
       <c r="F795">
-        <v>10300019002</v>
+        <v>10300016001</v>
       </c>
     </row>
     <row r="796">
       <c r="A796">
-        <v>10300019001226</v>
+        <v>10300019001225</v>
       </c>
       <c r="B796" t="str">
-        <v>هادیشهر</v>
+        <v>جلفا</v>
       </c>
       <c r="C796" t="str">
-        <v>هادیشهر</v>
+        <v>جلفا</v>
       </c>
       <c r="D796">
         <v>103</v>
@@ -16321,53 +16321,53 @@
     </row>
     <row r="797">
       <c r="A797">
-        <v>10300020001224</v>
+        <v>10300019001226</v>
       </c>
       <c r="B797" t="str">
-        <v>ملکان</v>
+        <v>هادیشهر</v>
       </c>
       <c r="C797" t="str">
-        <v>ملکان</v>
+        <v>هادیشهر</v>
       </c>
       <c r="D797">
         <v>103</v>
       </c>
       <c r="E797">
-        <v>10300020</v>
+        <v>10300019</v>
       </c>
       <c r="F797">
-        <v>10300020002</v>
+        <v>10300019002</v>
       </c>
     </row>
     <row r="798">
       <c r="A798">
-        <v>10300021001201</v>
+        <v>10300020001224</v>
       </c>
       <c r="B798" t="str">
-        <v>آذرشهر</v>
+        <v>ملکان</v>
       </c>
       <c r="C798" t="str">
-        <v>آذرشهر</v>
+        <v>ملکان</v>
       </c>
       <c r="D798">
         <v>103</v>
       </c>
       <c r="E798">
-        <v>10300021</v>
+        <v>10300020</v>
       </c>
       <c r="F798">
-        <v>10300021003</v>
+        <v>10300020002</v>
       </c>
     </row>
     <row r="799">
       <c r="A799">
-        <v>10300021001202</v>
+        <v>10300021001201</v>
       </c>
       <c r="B799" t="str">
-        <v>گوگان</v>
+        <v>آذرشهر</v>
       </c>
       <c r="C799" t="str">
-        <v>گوگان</v>
+        <v>آذرشهر</v>
       </c>
       <c r="D799">
         <v>103</v>
@@ -16376,18 +16376,18 @@
         <v>10300021</v>
       </c>
       <c r="F799">
-        <v>10300021001</v>
+        <v>10300021003</v>
       </c>
     </row>
     <row r="800">
       <c r="A800">
-        <v>10300021001203</v>
+        <v>10300021001202</v>
       </c>
       <c r="B800" t="str">
-        <v>ممقان</v>
+        <v>گوگان</v>
       </c>
       <c r="C800" t="str">
-        <v>ممقان</v>
+        <v>گوگان</v>
       </c>
       <c r="D800">
         <v>103</v>
@@ -16396,18 +16396,18 @@
         <v>10300021</v>
       </c>
       <c r="F800">
-        <v>10300021002</v>
+        <v>10300021001</v>
       </c>
     </row>
     <row r="801">
       <c r="A801">
-        <v>10300021002763</v>
+        <v>10300021001203</v>
       </c>
       <c r="B801" t="str">
-        <v>تیمورلو</v>
+        <v>ممقان</v>
       </c>
       <c r="C801" t="str">
-        <v>تیمورلو</v>
+        <v>ممقان</v>
       </c>
       <c r="D801">
         <v>103</v>
@@ -16416,38 +16416,38 @@
         <v>10300021</v>
       </c>
       <c r="F801">
-        <v>10300021001</v>
+        <v>10300021002</v>
       </c>
     </row>
     <row r="802">
       <c r="A802">
-        <v>10300022001204</v>
+        <v>10300021002763</v>
       </c>
       <c r="B802" t="str">
-        <v>اسکو</v>
+        <v>تیمورلو</v>
       </c>
       <c r="C802" t="str">
-        <v>اسکو</v>
+        <v>تیمورلو</v>
       </c>
       <c r="D802">
         <v>103</v>
       </c>
       <c r="E802">
-        <v>10300022</v>
+        <v>10300021</v>
       </c>
       <c r="F802">
-        <v>10300022002</v>
+        <v>10300021001</v>
       </c>
     </row>
     <row r="803">
       <c r="A803">
-        <v>10300022001205</v>
+        <v>10300022001204</v>
       </c>
       <c r="B803" t="str">
-        <v>ایلخچی</v>
+        <v>اسکو</v>
       </c>
       <c r="C803" t="str">
-        <v>ایلخچی</v>
+        <v>اسکو</v>
       </c>
       <c r="D803">
         <v>103</v>
@@ -16456,18 +16456,18 @@
         <v>10300022</v>
       </c>
       <c r="F803">
-        <v>10300022001</v>
+        <v>10300022002</v>
       </c>
     </row>
     <row r="804">
       <c r="A804">
-        <v>10300022002033</v>
+        <v>10300022001205</v>
       </c>
       <c r="B804" t="str">
-        <v>سهند</v>
+        <v>ایلخچی</v>
       </c>
       <c r="C804" t="str">
-        <v>سهند</v>
+        <v>ایلخچی</v>
       </c>
       <c r="D804">
         <v>103</v>
@@ -16476,38 +16476,38 @@
         <v>10300022</v>
       </c>
       <c r="F804">
-        <v>10300022002</v>
+        <v>10300022001</v>
       </c>
     </row>
     <row r="805">
       <c r="A805">
-        <v>10300024002142</v>
+        <v>10300022002033</v>
       </c>
       <c r="B805" t="str">
-        <v>ورزقان</v>
+        <v>سهند</v>
       </c>
       <c r="C805" t="str">
-        <v>ورزقان</v>
+        <v>سهند</v>
       </c>
       <c r="D805">
         <v>103</v>
       </c>
       <c r="E805">
-        <v>10300024</v>
+        <v>10300022</v>
       </c>
       <c r="F805">
-        <v>10300024002</v>
+        <v>10300022002</v>
       </c>
     </row>
     <row r="806">
       <c r="A806">
-        <v>10300024002398</v>
+        <v>10300024002142</v>
       </c>
       <c r="B806" t="str">
-        <v>خاروانا</v>
+        <v>ورزقان</v>
       </c>
       <c r="C806" t="str">
-        <v>خاروانا</v>
+        <v>ورزقان</v>
       </c>
       <c r="D806">
         <v>103</v>
@@ -16516,38 +16516,38 @@
         <v>10300024</v>
       </c>
       <c r="F806">
-        <v>10300024001</v>
+        <v>10300024002</v>
       </c>
     </row>
     <row r="807">
       <c r="A807">
-        <v>10300026002332</v>
+        <v>10300024002398</v>
       </c>
       <c r="B807" t="str">
-        <v>خمارلو</v>
+        <v>خاروانا</v>
       </c>
       <c r="C807" t="str">
-        <v>خمارلو</v>
+        <v>خاروانا</v>
       </c>
       <c r="D807">
         <v>103</v>
       </c>
       <c r="E807">
-        <v>10300026</v>
+        <v>10300024</v>
       </c>
       <c r="F807">
-        <v>10300026001</v>
+        <v>10300024001</v>
       </c>
     </row>
     <row r="808">
       <c r="A808">
-        <v>10300026002944</v>
+        <v>10300026002332</v>
       </c>
       <c r="B808" t="str">
-        <v>عاشقلو</v>
+        <v>خمارلو</v>
       </c>
       <c r="C808" t="str">
-        <v>عاشقلو</v>
+        <v>خمارلو</v>
       </c>
       <c r="D808">
         <v>103</v>
@@ -16556,18 +16556,18 @@
         <v>10300026</v>
       </c>
       <c r="F808">
-        <v>10300026003</v>
+        <v>10300026001</v>
       </c>
     </row>
     <row r="809">
       <c r="A809">
-        <v>10300026002945</v>
+        <v>10300026002944</v>
       </c>
       <c r="B809" t="str">
-        <v>لاریجان</v>
+        <v>عاشقلو</v>
       </c>
       <c r="C809" t="str">
-        <v>لاریجان</v>
+        <v>عاشقلو</v>
       </c>
       <c r="D809">
         <v>103</v>
@@ -16576,67 +16576,67 @@
         <v>10300026</v>
       </c>
       <c r="F809">
-        <v>10300026002</v>
+        <v>10300026003</v>
       </c>
     </row>
     <row r="810">
       <c r="A810">
-        <v>10300027002294</v>
+        <v>10300026002945</v>
       </c>
       <c r="B810" t="str">
-        <v>هوراند</v>
+        <v>لاریجان</v>
       </c>
       <c r="C810" t="str">
-        <v>هوراند</v>
+        <v>لاریجان</v>
       </c>
       <c r="D810">
         <v>103</v>
       </c>
       <c r="E810">
-        <v>10300027</v>
+        <v>10300026</v>
       </c>
       <c r="F810">
-        <v>10300027001</v>
+        <v>10300026002</v>
       </c>
     </row>
     <row r="811">
       <c r="A811">
-        <v>10300028002296</v>
+        <v>10300027002294</v>
       </c>
       <c r="B811" t="str">
-        <v>لیلان</v>
+        <v>هوراند</v>
       </c>
       <c r="C811" t="str">
-        <v>لیلان</v>
+        <v>هوراند</v>
       </c>
       <c r="D811">
         <v>103</v>
       </c>
       <c r="E811">
-        <v>10300028</v>
+        <v>10300027</v>
       </c>
       <c r="F811">
-        <v>10300028001</v>
+        <v>10300027001</v>
       </c>
     </row>
     <row r="812">
       <c r="A812">
-        <v>10300029002144</v>
+        <v>10300028002296</v>
       </c>
       <c r="B812" t="str">
-        <v>ترکمانچای</v>
+        <v>لیلان</v>
       </c>
       <c r="C812" t="str">
-        <v>ترکمانچای</v>
+        <v>لیلان</v>
       </c>
       <c r="D812">
         <v>103</v>
       </c>
       <c r="E812">
-        <v>10300029</v>
+        <v>10300028</v>
       </c>
       <c r="F812">
-        <v>10300029001</v>
+        <v>10300028001</v>
       </c>
     </row>
     <row r="813">

</xml_diff>